<commit_message>
fix(dxf): disegno solo per l'amministratore, errori gestiti
- La voce 'Disegno DXF' compare solo con il ruolo admin; la guida non lo
  promette piu' ai clienti.
- Errore nella generazione: messaggio invece di un clic muto; paneConfigs
  con elementi vuoti non manda in errore.
- Titolo del cassonetto senza 'N ANTE', come nel PDF; spazio per i titoli
  lunghi fra un serramento e l'altro.
- Modello Excel: la data si scrive a mano (con OGGI() cambiava a ogni
  apertura).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/modelli/modello-preventivo-infissi.xlsx
+++ b/public/modelli/modello-preventivo-infissi.xlsx
@@ -666,10 +666,7 @@
           <t>Data</t>
         </is>
       </c>
-      <c r="K3" s="6">
-        <f>TODAY()</f>
-        <v/>
-      </c>
+      <c r="K3" s="6" t="n"/>
     </row>
     <row r="4">
       <c r="I4" s="4" t="inlineStr">

</xml_diff>